<commit_message>
Add three valid L-length test cases
</commit_message>
<xml_diff>
--- a/test_automation/IT23687882_Assignment 1 - Test cases_FIXED.xlsx
+++ b/test_automation/IT23687882_Assignment 1 - Test cases_FIXED.xlsx
@@ -367,24 +367,20 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>oya ada campus yanawada?</t>
+          <t>oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada?</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>ඔයා අද කැම්පස් යනවාද?</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr">
-        <is>
-          <t>ඔයා අද campus යනවද?</t>
-        </is>
-      </c>
+          <t>??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ??????</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -451,24 +447,20 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>denmafileekayawanna.</t>
+          <t>denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>දැන්ම file එක යවන්න.</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>දැන්මෆීලීයවන්න.</t>
-        </is>
-      </c>
+          <t>????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????.</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -619,24 +611,20 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>matapoddakudawkaranna.</t>
+          <t>matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna.</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>මට පොඩ්ඩක් උදව් කරන්න.</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr">
-        <is>
-          <t>මට පොඩ්ඩක්උඩව්කරන්න.</t>
-        </is>
-      </c>
+          <t>?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????.</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>FAIL</t>

</xml_diff>

<commit_message>
Fill L-case actual output placeholders
</commit_message>
<xml_diff>
--- a/test_automation/IT23687882_Assignment 1 - Test cases_FIXED.xlsx
+++ b/test_automation/IT23687882_Assignment 1 - Test cases_FIXED.xlsx
@@ -372,15 +372,19 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada? oya ada campus yanawada?</t>
+          <t>mama ada ude campus yanakota bus eka godak parakku una, eth mama assignment eka submit karanna kalin library ekata giya, eeta passe yaluwo ekka group discussion ekak dala project eke authentication part eka explain kara, rathriyata gedara awith thawa test cases tika balala code eka run karala errors hadanna hithuwa, meka hariyata karoth marks hodata ganna puluwan kiyala mata sure kiyala hithanawa.</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ?????? ??? ?? ??????? ??????</t>
-        </is>
-      </c>
-      <c r="E2" s="1" t="inlineStr"/>
+          <t>මම අද උදේ කැම්පස් යනකොට බස් එක ගොඩක් පරක්කු වුණා, එත් මම අසයින්මන්ට් එක සබ්මිට් කරන්න කලින් ලයිබ්‍රරි එකට ගියා, ඊට පස්සේ යාලුවෝ එක්ක ග්‍රූප් ඩිස්කෂන් එකක් දාලා ප්‍රොජෙක්ට් එකේ ඔතෙන්ටිකේෂන් පාර්ට් එක එක්ස්ප්ලේන් කළා, රෑට ගෙදර ඇවිත් තව ටෙස්ට් කේස් ටික බලලා කෝඩ් එක රන් කරලා එරර්ස් හදන්න හිතුවා, මේක හරියට කළොත් මාක්ස් හොඳට ගන්න පුළුවන් කියලා මට ෂුවර් කියලා හිතනවා.</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>[No output returned for this L input]</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -452,15 +456,19 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna. denmafileekayawanna.</t>
+          <t>ape smart campus system eke users lata login wenna email password wage normal method ekak thiyenawa, google oauth2 login ekath add karala thiyenawa, admin kenek resources create update delete karanna puluwan, students lata facilities book karanna puluwan, notification panel eken status updates balanna puluwan, ehema unaama campus work eka godak lesi wenawa meka project ekata hoda value ekak denawa.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????. ????? file ?? ?????.</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr"/>
+          <t>අපේ ස්මාර්ට් කැම්පස් සිස්ටම් එකේ යූසර්ස්ලාට ලොගින් වෙන්න ඊමේල් පාස්වර්ඩ් වගේ නොර්මල් මෙතඩ් එකක් තියෙනවා, ගූගල් ඕඕත් ටූ ලොගින් එකත් ඇඩ් කරලා තියෙනවා, ඇඩ්මින් කෙනෙක්ට රිසෝසස් ක්‍රියේට් අප්ඩේට් ඩිලිට් කරන්න පුළුවන්, ස්ටුඩන්ට්ස්ලාට ෆැසිලිටීස් බුක් කරන්න පුළුවන්, නොටිෆිකේෂන් පැනල් එකෙන් ස්ටේටස් අප්ඩේට්ස් බලන්න පුළුවන්, එහෙම වුණාම කැම්පස් වර්ක් එක ගොඩක් ලේසි වෙනවා මේක ප්‍රොජෙක්ට් එකට හොඳ වැලියු එකක් දෙනවා.</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>[No output returned for this L input]</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>FAIL</t>
@@ -616,15 +624,19 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna. matapoddakudawkaranna.</t>
+          <t>mata database indexing lesson eka mula idan tikak amarui wage hithuna, namuth dense index sparse index clustered index unclustered index kiyala wenama note ekak hadagaththama concept eka theruna, hash file organization wala static hashing dynamic hashing local depth global depth gana api viva ekata ready wenna one, sir ahuwoth short answer ekak denna puluwan e nisa mata dan bayak nathiwa answer karanna puluwan.</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????. ?? ??????? ???? ?????.</t>
-        </is>
-      </c>
-      <c r="E8" s="1" t="inlineStr"/>
+          <t>මට ඩේටාබේස් ඉන්ඩෙක්සින් ලෙස්න් එක මුල ඉඳන් ටිකක් අමාරුයි වගේ හිතුණා, නමුත් ඩෙන්ස් ඉන්ඩෙක්ස් ස්පාර්ස් ඉන්ඩෙක්ස් ක්ලස්ටර්ඩ් ඉන්ඩෙක්ස් අන්ක්ලස්ටර්ඩ් ඉන්ඩෙක්ස් කියලා වෙනම නෝට් එකක් හදාගත්තම කොන්සෙප්ට් එක තේරුණා, හැෂ් ෆයිල් ඕගනයිසේෂන් වල ස්ටැටික් හැෂින් ඩයිනමික් හැෂින් ලෝකල් ඩෙප්ත් ග්ලෝබල් ඩෙප්ත් ගැන අපි වයිවා එකට රෙඩි වෙන්න ඕන, සර් ඇහුවොත් ෂෝර්ට් ආන්සර් එකක් දෙන්න පුළුවන් ඒ නිසා මට දැන් බයක් නැතිව ආන්සර් කරන්න පුළුවන්.</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>[No output returned for this L input]</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>FAIL</t>

</xml_diff>

<commit_message>
Capture actual outputs for L-length test rows
</commit_message>
<xml_diff>
--- a/test_automation/IT23687882_Assignment 1 - Test cases_FIXED.xlsx
+++ b/test_automation/IT23687882_Assignment 1 - Test cases_FIXED.xlsx
@@ -382,7 +382,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>[No output returned for this L input]</t>
+          <t>මම අද උදේ campus යනකොට bus එක ගොඩක් පරක්කු උනා, ඒත් මම assignment එක submit කරන්න කලින් library එකට ගියා, ඊට පස්සේ යාලුවෝ එක්ක group discussion එකක් දාලා project එකේ authentication part එක explain කරා, රාත්‍රියට ගෙදර ඇවිත් තව ටෙස්ට් කේස්ස් ටික බලලා කෝඩ් එක රූන් කරලා එර්රෝර්ස් හදන්න හිතුවා, මේක හරියට කරොත් marks හොදට ගන්න පුළුවන් කියලා මට sure කියලා හිතනවා.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>[No output returned for this L input]</t>
+          <t>අපේ smart campus system එකේ users ලාට login වෙන්න email password වගේ normal method එකක් තියෙනවා, google ඕඅඋත්2 login එකත් add කරලා තියෙනවා, admin කෙනෙක් resources create update delete කරන්න පුළුවන්, students ලාට facilities book කරන්න පුළුවන්, notification panel එකෙන් status updates බලන්න පුළුවන්, එහෙම උනාම campus work එක ගොඩක් ලේසි වෙනවා මේක project එකට හොඳ value එකක් දෙනවා.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>[No output returned for this L input]</t>
+          <t>මට database indexing lesson එක මුල ඉදන් ටිකක් අමාරුයි වගේ හිතුණා, නමුත් දැන්සේ index sparse index clustered index unclustered index කියලා වෙනම note එකක් හදාගත්තම concept එක තේරුනා, hash file organization වල static hashing dynamic hashing local දෙප්ත් global දෙප්ත් ගැන අපි viva එකට ready වෙන්න ඕනේ, sir ඇහුවොත් short answer එකක් දෙන්න පුළුවන් ඒ නිසා මට දැන් බයක් නැතිව answer කරන්න පුළුවන්.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>